<commit_message>
Deployed 98a4a0d with MkDocs version: 1.0.4
</commit_message>
<xml_diff>
--- a/images/Employment.xlsx
+++ b/images/Employment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simon.rhee\Desktop\gitpage\docs\images\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F78114-D07F-4740-88B9-80D805361B9B}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{579B77A2-E87A-40F5-88EB-058681E70F48}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{C666FD2C-32AC-43EC-BEA7-25CE32E05CBB}"/>
   </bookViews>
@@ -1061,9 +1061,7 @@
       <a:schemeClr val="bg1"/>
     </a:solidFill>
     <a:ln w="31750" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1"/>
-      </a:solidFill>
+      <a:noFill/>
       <a:round/>
     </a:ln>
     <a:effectLst/>
@@ -1695,9 +1693,7 @@
       <a:schemeClr val="bg1"/>
     </a:solidFill>
     <a:ln w="31750" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1"/>
-      </a:solidFill>
+      <a:noFill/>
       <a:round/>
     </a:ln>
     <a:effectLst/>

</xml_diff>